<commit_message>
diabetes python was updated
</commit_message>
<xml_diff>
--- a/steps.xlsx
+++ b/steps.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianaoliveira/Desktop/DataScience/Diabetes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88B82877-438E-194C-90FE-06D87CDD58AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B1326D8-6CA5-3542-B7ED-B6EA65764BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{F4A15B66-7D43-9342-9E39-E833C261D95C}"/>
+    <workbookView xWindow="38560" yWindow="660" windowWidth="33880" windowHeight="20540" activeTab="1" xr2:uid="{F4A15B66-7D43-9342-9E39-E833C261D95C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="todo" sheetId="1" r:id="rId1"/>
+    <sheet name="3" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="87">
   <si>
     <t>Step</t>
   </si>
@@ -319,6 +320,132 @@
   </si>
   <si>
     <t>Public portfolio</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Tools</t>
+  </si>
+  <si>
+    <t>Example Code</t>
+  </si>
+  <si>
+    <t>Why It Matters</t>
+  </si>
+  <si>
+    <t>Preview Data</t>
+  </si>
+  <si>
+    <t>Look at first/last rows</t>
+  </si>
+  <si>
+    <t>Pandas</t>
+  </si>
+  <si>
+    <r>
+      <t>df.head()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>df.tail()</t>
+    </r>
+  </si>
+  <si>
+    <t>Quickly understand structure</t>
+  </si>
+  <si>
+    <t>Shape of Data</t>
+  </si>
+  <si>
+    <t>Check rows &amp; columns</t>
+  </si>
+  <si>
+    <t>df.shape</t>
+  </si>
+  <si>
+    <t>Know dataset size</t>
+  </si>
+  <si>
+    <t>Column Info</t>
+  </si>
+  <si>
+    <t>Check data types &amp; nulls</t>
+  </si>
+  <si>
+    <t>df.info()</t>
+  </si>
+  <si>
+    <t>Detect wrong types &amp; missing values</t>
+  </si>
+  <si>
+    <t>Summary Stats</t>
+  </si>
+  <si>
+    <t>Get mean, std, min, max</t>
+  </si>
+  <si>
+    <t>df.describe()</t>
+  </si>
+  <si>
+    <t>Spot unusual values</t>
+  </si>
+  <si>
+    <t>Missing Values</t>
+  </si>
+  <si>
+    <t>Count missing/nulls</t>
+  </si>
+  <si>
+    <t>df.isnull().sum()</t>
+  </si>
+  <si>
+    <t>Identify cleaning needs</t>
+  </si>
+  <si>
+    <t>Zero Values Check</t>
+  </si>
+  <si>
+    <t>Detect invalid zeros (important here!)</t>
+  </si>
+  <si>
+    <t>(df == 0).sum()</t>
+  </si>
+  <si>
+    <t>Some columns shouldn't be zero</t>
+  </si>
+  <si>
+    <t>Unique Values</t>
+  </si>
+  <si>
+    <t>Check categories (e.g., Outcome)</t>
+  </si>
+  <si>
+    <t>df['Outcome'].value_counts()</t>
+  </si>
+  <si>
+    <t>Understand target balance</t>
   </si>
 </sst>
 </file>
@@ -376,7 +503,62 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -387,6 +569,36 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0A810063-40F0-8C44-857F-9FB26D52C5D1}" name="Table2" displayName="Table2" ref="A1:F13" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:F13" xr:uid="{0A810063-40F0-8C44-857F-9FB26D52C5D1}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{9B43C5FC-5853-E94C-B6E9-247E6984FF12}" name="Step"/>
+    <tableColumn id="2" xr3:uid="{666BAAE1-BBB2-7149-A9A7-236CF54D8249}" name="Phase"/>
+    <tableColumn id="3" xr3:uid="{AD2D07A8-31B5-2141-93E4-1727076BCBEB}" name="What You Do"/>
+    <tableColumn id="4" xr3:uid="{F0C13477-85E2-9E48-9FAE-4D0FDA4F7B1E}" name="Tools / Technologies"/>
+    <tableColumn id="5" xr3:uid="{A25AF6DB-93A8-DA4D-A3F0-10F0138E85B0}" name="Output"/>
+    <tableColumn id="6" xr3:uid="{F246AD3D-FB1B-D740-BCFD-38B97FA1F1DC}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C573F72D-B02B-E746-94D8-0B40D19A651F}" name="Table3" displayName="Table3" ref="A1:F8" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:F8" xr:uid="{C573F72D-B02B-E746-94D8-0B40D19A651F}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{7DC519C7-CE93-9543-8EF0-F412BE37011C}" name="Task"/>
+    <tableColumn id="2" xr3:uid="{B4923D26-0217-4649-A8B6-C8C715F1D3FA}" name="What You Do"/>
+    <tableColumn id="3" xr3:uid="{A6657E80-6A98-4946-A08A-917D94195FF4}" name="Tools"/>
+    <tableColumn id="4" xr3:uid="{17B2F1CD-2F5F-8E4B-B751-E7125F01419A}" name="Example Code" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{E1A21EDC-C532-0A42-963D-55286B62E67F}" name="Why It Matters"/>
+    <tableColumn id="6" xr3:uid="{BC0E6A16-13B4-2C48-81C5-E5932B1846B1}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -706,16 +918,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{625A0ED6-9AA2-9349-B3F0-83632E95E1DE}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="41.33203125" customWidth="1"/>
     <col min="3" max="3" width="53" customWidth="1"/>
     <col min="4" max="4" width="32.6640625" customWidth="1"/>
-    <col min="5" max="5" width="24.6640625" customWidth="1"/>
+    <col min="5" max="5" width="22.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -731,8 +943,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -748,8 +963,11 @@
       <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -765,8 +983,11 @@
       <c r="E3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -783,7 +1004,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -800,7 +1021,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -817,7 +1038,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -834,7 +1055,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -851,7 +1072,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -868,7 +1089,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -885,7 +1106,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -902,7 +1123,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -919,7 +1140,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -938,5 +1159,188 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25619793-E213-8D48-98F7-41635E2B4070}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" customWidth="1"/>
+    <col min="4" max="5" width="35.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataConsolidate/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>